<commit_message>
Add new Excel file for customer issue documentation
- Created a new Excel file named 'lampiran_b_masalah_pelanggan.xlsx' to document customer issues.
- The file includes multiple sheets and structured data for better organization and tracking of customer problems.
</commit_message>
<xml_diff>
--- a/Detail & Kalkulasi Rendy Audio.xlsx
+++ b/Detail & Kalkulasi Rendy Audio.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kelinci\Downloads\TA\Steven\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kelinci\Downloads\Web_Steven\audio_match_api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3893FA55-5457-40B3-89CC-D1D6E8B95C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CA0747-49AB-4DB7-A0D5-6663E9148966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1802,15 +1802,14 @@
   <dimension ref="A1:F151"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="38" customWidth="1"/>
-    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="35.5546875" customWidth="1"/>
+    <col min="3" max="3" width="6.77734375" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" customWidth="1"/>
+    <col min="5" max="6" width="35.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1830,7 +1829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1870,7 +1869,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1930,7 +1929,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -1970,7 +1969,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
@@ -2010,7 +2009,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -2050,7 +2049,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>30</v>
       </c>
@@ -2130,7 +2129,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>42</v>
       </c>
@@ -2150,7 +2149,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -2170,7 +2169,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>42</v>
       </c>
@@ -2210,7 +2209,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>42</v>
       </c>
@@ -2230,7 +2229,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>54</v>
       </c>
@@ -2270,7 +2269,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>54</v>
       </c>
@@ -2290,7 +2289,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>54</v>
       </c>
@@ -2310,7 +2309,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>54</v>
       </c>
@@ -2550,7 +2549,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>90</v>
       </c>
@@ -2570,7 +2569,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>90</v>
       </c>
@@ -2590,7 +2589,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>90</v>
       </c>
@@ -2610,7 +2609,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>90</v>
       </c>
@@ -2670,7 +2669,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>102</v>
       </c>
@@ -2690,7 +2689,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>102</v>
       </c>
@@ -2710,7 +2709,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>102</v>
       </c>
@@ -2750,7 +2749,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>114</v>
       </c>
@@ -2770,7 +2769,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>114</v>
       </c>
@@ -2790,7 +2789,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>114</v>
       </c>
@@ -2810,7 +2809,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>114</v>
       </c>
@@ -2910,7 +2909,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>126</v>
       </c>
@@ -2930,7 +2929,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>138</v>
       </c>
@@ -2970,7 +2969,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>138</v>
       </c>
@@ -3010,7 +3009,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>138</v>
       </c>
@@ -3210,7 +3209,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>161</v>
       </c>
@@ -3290,7 +3289,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>173</v>
       </c>
@@ -3310,7 +3309,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>173</v>
       </c>
@@ -3390,7 +3389,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>184</v>
       </c>
@@ -3430,7 +3429,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>196</v>
       </c>
@@ -4310,7 +4309,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>288</v>
       </c>
@@ -4350,7 +4349,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>300</v>
       </c>
@@ -4450,7 +4449,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
         <v>312</v>
       </c>
@@ -4550,7 +4549,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>324</v>
       </c>
@@ -4590,7 +4589,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>324</v>
       </c>
@@ -4650,7 +4649,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
         <v>335</v>
       </c>
@@ -4710,7 +4709,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>335</v>
       </c>
@@ -4750,7 +4749,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>346</v>
       </c>
@@ -4810,7 +4809,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A151" s="5" t="s">
         <v>346</v>
       </c>
@@ -4833,7 +4832,7 @@
   </sheetData>
   <autoFilter ref="A1:F151" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4927,7 +4926,7 @@
         <v>369</v>
       </c>
       <c r="L2" s="9">
-        <f>(IF(D2&gt;0,1,0)+IF(E2&gt;0,1,0)+IF(F2&gt;0,1,0)+IF(G2&gt;0,1,0)+IF(H2&gt;0,1,0))/5</f>
+        <f t="shared" ref="L2:L31" si="1">(IF(D2&gt;0,1,0)+IF(E2&gt;0,1,0)+IF(F2&gt;0,1,0)+IF(G2&gt;0,1,0)+IF(H2&gt;0,1,0))/5</f>
         <v>0.2</v>
       </c>
     </row>
@@ -4967,7 +4966,7 @@
         <v>372</v>
       </c>
       <c r="L3" s="10">
-        <f>(IF(D3&gt;0,1,0)+IF(E3&gt;0,1,0)+IF(F3&gt;0,1,0)+IF(G3&gt;0,1,0)+IF(H3&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5007,7 +5006,7 @@
         <v>375</v>
       </c>
       <c r="L4" s="9">
-        <f>(IF(D4&gt;0,1,0)+IF(E4&gt;0,1,0)+IF(F4&gt;0,1,0)+IF(G4&gt;0,1,0)+IF(H4&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
     </row>
@@ -5047,7 +5046,7 @@
         <v>378</v>
       </c>
       <c r="L5" s="10">
-        <f>(IF(D5&gt;0,1,0)+IF(E5&gt;0,1,0)+IF(F5&gt;0,1,0)+IF(G5&gt;0,1,0)+IF(H5&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5087,7 +5086,7 @@
         <v>381</v>
       </c>
       <c r="L6" s="9">
-        <f>(IF(D6&gt;0,1,0)+IF(E6&gt;0,1,0)+IF(F6&gt;0,1,0)+IF(G6&gt;0,1,0)+IF(H6&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5127,7 +5126,7 @@
         <v>381</v>
       </c>
       <c r="L7" s="10">
-        <f>(IF(D7&gt;0,1,0)+IF(E7&gt;0,1,0)+IF(F7&gt;0,1,0)+IF(G7&gt;0,1,0)+IF(H7&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5167,7 +5166,7 @@
         <v>384</v>
       </c>
       <c r="L8" s="9">
-        <f>(IF(D8&gt;0,1,0)+IF(E8&gt;0,1,0)+IF(F8&gt;0,1,0)+IF(G8&gt;0,1,0)+IF(H8&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
     </row>
@@ -5207,7 +5206,7 @@
         <v>386</v>
       </c>
       <c r="L9" s="10">
-        <f>(IF(D9&gt;0,1,0)+IF(E9&gt;0,1,0)+IF(F9&gt;0,1,0)+IF(G9&gt;0,1,0)+IF(H9&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
     </row>
@@ -5247,7 +5246,7 @@
         <v>388</v>
       </c>
       <c r="L10" s="9">
-        <f>(IF(D10&gt;0,1,0)+IF(E10&gt;0,1,0)+IF(F10&gt;0,1,0)+IF(G10&gt;0,1,0)+IF(H10&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -5287,7 +5286,7 @@
         <v>386</v>
       </c>
       <c r="L11" s="10">
-        <f>(IF(D11&gt;0,1,0)+IF(E11&gt;0,1,0)+IF(F11&gt;0,1,0)+IF(G11&gt;0,1,0)+IF(H11&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
     </row>
@@ -5327,7 +5326,7 @@
         <v>386</v>
       </c>
       <c r="L12" s="9">
-        <f>(IF(D12&gt;0,1,0)+IF(E12&gt;0,1,0)+IF(F12&gt;0,1,0)+IF(G12&gt;0,1,0)+IF(H12&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
     </row>
@@ -5367,7 +5366,7 @@
         <v>391</v>
       </c>
       <c r="L13" s="10">
-        <f>(IF(D13&gt;0,1,0)+IF(E13&gt;0,1,0)+IF(F13&gt;0,1,0)+IF(G13&gt;0,1,0)+IF(H13&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -5407,7 +5406,7 @@
         <v>393</v>
       </c>
       <c r="L14" s="9">
-        <f>(IF(D14&gt;0,1,0)+IF(E14&gt;0,1,0)+IF(F14&gt;0,1,0)+IF(G14&gt;0,1,0)+IF(H14&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5447,7 +5446,7 @@
         <v>388</v>
       </c>
       <c r="L15" s="10">
-        <f>(IF(D15&gt;0,1,0)+IF(E15&gt;0,1,0)+IF(F15&gt;0,1,0)+IF(G15&gt;0,1,0)+IF(H15&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -5487,7 +5486,7 @@
         <v>397</v>
       </c>
       <c r="L16" s="9">
-        <f>(IF(D16&gt;0,1,0)+IF(E16&gt;0,1,0)+IF(F16&gt;0,1,0)+IF(G16&gt;0,1,0)+IF(H16&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -5527,7 +5526,7 @@
         <v>399</v>
       </c>
       <c r="L17" s="10">
-        <f>(IF(D17&gt;0,1,0)+IF(E17&gt;0,1,0)+IF(F17&gt;0,1,0)+IF(G17&gt;0,1,0)+IF(H17&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -5567,7 +5566,7 @@
         <v>401</v>
       </c>
       <c r="L18" s="9">
-        <f>(IF(D18&gt;0,1,0)+IF(E18&gt;0,1,0)+IF(F18&gt;0,1,0)+IF(G18&gt;0,1,0)+IF(H18&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -5607,7 +5606,7 @@
         <v>388</v>
       </c>
       <c r="L19" s="10">
-        <f>(IF(D19&gt;0,1,0)+IF(E19&gt;0,1,0)+IF(F19&gt;0,1,0)+IF(G19&gt;0,1,0)+IF(H19&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -5647,7 +5646,7 @@
         <v>401</v>
       </c>
       <c r="L20" s="9">
-        <f>(IF(D20&gt;0,1,0)+IF(E20&gt;0,1,0)+IF(F20&gt;0,1,0)+IF(G20&gt;0,1,0)+IF(H20&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -5687,7 +5686,7 @@
         <v>378</v>
       </c>
       <c r="L21" s="10">
-        <f>(IF(D21&gt;0,1,0)+IF(E21&gt;0,1,0)+IF(F21&gt;0,1,0)+IF(G21&gt;0,1,0)+IF(H21&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5727,7 +5726,7 @@
         <v>405</v>
       </c>
       <c r="L22" s="9">
-        <f>(IF(D22&gt;0,1,0)+IF(E22&gt;0,1,0)+IF(F22&gt;0,1,0)+IF(G22&gt;0,1,0)+IF(H22&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -5767,7 +5766,7 @@
         <v>378</v>
       </c>
       <c r="L23" s="10">
-        <f>(IF(D23&gt;0,1,0)+IF(E23&gt;0,1,0)+IF(F23&gt;0,1,0)+IF(G23&gt;0,1,0)+IF(H23&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5807,7 +5806,7 @@
         <v>381</v>
       </c>
       <c r="L24" s="9">
-        <f>(IF(D24&gt;0,1,0)+IF(E24&gt;0,1,0)+IF(F24&gt;0,1,0)+IF(G24&gt;0,1,0)+IF(H24&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
     </row>
@@ -5847,7 +5846,7 @@
         <v>401</v>
       </c>
       <c r="L25" s="10">
-        <f>(IF(D25&gt;0,1,0)+IF(E25&gt;0,1,0)+IF(F25&gt;0,1,0)+IF(G25&gt;0,1,0)+IF(H25&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -5887,7 +5886,7 @@
         <v>401</v>
       </c>
       <c r="L26" s="9">
-        <f>(IF(D26&gt;0,1,0)+IF(E26&gt;0,1,0)+IF(F26&gt;0,1,0)+IF(G26&gt;0,1,0)+IF(H26&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -5927,7 +5926,7 @@
         <v>410</v>
       </c>
       <c r="L27" s="10">
-        <f>(IF(D27&gt;0,1,0)+IF(E27&gt;0,1,0)+IF(F27&gt;0,1,0)+IF(G27&gt;0,1,0)+IF(H27&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -5967,7 +5966,7 @@
         <v>401</v>
       </c>
       <c r="L28" s="9">
-        <f>(IF(D28&gt;0,1,0)+IF(E28&gt;0,1,0)+IF(F28&gt;0,1,0)+IF(G28&gt;0,1,0)+IF(H28&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
@@ -6007,7 +6006,7 @@
         <v>410</v>
       </c>
       <c r="L29" s="10">
-        <f>(IF(D29&gt;0,1,0)+IF(E29&gt;0,1,0)+IF(F29&gt;0,1,0)+IF(G29&gt;0,1,0)+IF(H29&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -6047,7 +6046,7 @@
         <v>410</v>
       </c>
       <c r="L30" s="9">
-        <f>(IF(D30&gt;0,1,0)+IF(E30&gt;0,1,0)+IF(F30&gt;0,1,0)+IF(G30&gt;0,1,0)+IF(H30&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
     </row>
@@ -6087,7 +6086,7 @@
         <v>414</v>
       </c>
       <c r="L31" s="10">
-        <f>(IF(D31&gt;0,1,0)+IF(E31&gt;0,1,0)+IF(F31&gt;0,1,0)+IF(G31&gt;0,1,0)+IF(H31&gt;0,1,0))/5</f>
+        <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
     </row>
@@ -6103,20 +6102,18 @@
   <dimension ref="A1:AN31"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="1" max="1" width="5.21875" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="7" width="3.5546875" customWidth="1"/>
-    <col min="8" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.6640625" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13" hidden="1" customWidth="1"/>
+    <col min="3" max="7" width="3.5546875" hidden="1" customWidth="1"/>
+    <col min="8" max="12" width="11.6640625" hidden="1" customWidth="1"/>
+    <col min="13" max="14" width="13" hidden="1" customWidth="1"/>
     <col min="15" max="17" width="13" customWidth="1"/>
     <col min="18" max="19" width="13" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="13" customWidth="1"/>
     <col min="21" max="21" width="13" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="18.33203125" customWidth="1"/>
+    <col min="22" max="22" width="13.5546875" customWidth="1"/>
     <col min="23" max="23" width="11.109375" customWidth="1"/>
-    <col min="24" max="24" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.5546875" customWidth="1"/>
     <col min="25" max="25" width="11.109375" customWidth="1"/>
     <col min="36" max="40" width="8.6640625" customWidth="1"/>
   </cols>
@@ -6292,7 +6289,7 @@
         <v>1</v>
       </c>
       <c r="V2" s="2" t="str">
-        <f t="shared" ref="V2:X31" si="6">CONCATENATE(LEFT(M2,6)," / ",LEFT(T2,6))</f>
+        <f t="shared" ref="V2:V31" si="6">CONCATENATE(LEFT(M2,6)," / ",LEFT(T2,6))</f>
         <v>0,5 / 1</v>
       </c>
       <c r="W2" s="9">

</xml_diff>